<commit_message>
vault backup: 2026-04-28 10:35:28
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model_balance_test.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model_balance_test.xlsx
@@ -14857,67 +14857,67 @@
         <v/>
       </c>
       <c r="R15" s="4">
-        <f>-('QTR BS'!O5-'QTR BS'!N5)-('QTR BS'!O8-'QTR BS'!N8)-('QTR BS'!O10-'QTR BS'!N10)-('QTR BS'!O12-'QTR BS'!N12)-('QTR BS'!O15-'QTR BS'!N15)-('QTR BS'!O17-'QTR BS'!N17)+('QTR BS'!O22-'QTR BS'!N22)+('QTR BS'!O25-'QTR BS'!N25)+('QTR BS'!O26-'QTR BS'!N26)+('QTR BS'!O27-'QTR BS'!N27)+('QTR BS'!O28-'QTR BS'!N28)+('QTR BS'!O31-'QTR BS'!N31)+('QTR BS'!O32-'QTR BS'!N32)+('QTR BS'!O35-'QTR BS'!N35)+('QTR BS'!O36-'QTR BS'!N36)-('QTR BS'!O3-'QTR BS'!N3)-('QTR BS'!O13-'QTR BS'!N13)-('QTR BS'!O14-'QTR BS'!N14)+('QTR BS'!O33-'QTR BS'!N33)+('QTR BS'!O34-'QTR BS'!N34)</f>
+        <f>-('QTR BS'!O5-'QTR BS'!N5)-('QTR BS'!O8-'QTR BS'!N8)-('QTR BS'!O10-'QTR BS'!N10)-('QTR BS'!O12-'QTR BS'!N12)-('QTR BS'!O15-'QTR BS'!N15)-('QTR BS'!O17-'QTR BS'!N17)+('QTR BS'!O22-'QTR BS'!N22)+('QTR BS'!O25-'QTR BS'!N25)+('QTR BS'!O26-'QTR BS'!N26)+('QTR BS'!O27-'QTR BS'!N27)+('QTR BS'!O28-'QTR BS'!N28)+('QTR BS'!O31-'QTR BS'!N31)+('QTR BS'!O32-'QTR BS'!N32)+('QTR BS'!O35-'QTR BS'!N35)+('QTR BS'!O36-'QTR BS'!N36)-('QTR BS'!O3-'QTR BS'!N3)-('QTR BS'!O13-'QTR BS'!N13)-('QTR BS'!O14-'QTR BS'!N14)+('QTR BS'!O23-'QTR BS'!N23)+('QTR BS'!O33-'QTR BS'!N33)+('QTR BS'!O34-'QTR BS'!N34)</f>
         <v/>
       </c>
       <c r="S15" s="4">
-        <f>-('QTR BS'!P5-'QTR BS'!O5)-('QTR BS'!P8-'QTR BS'!O8)-('QTR BS'!P10-'QTR BS'!O10)-('QTR BS'!P12-'QTR BS'!O12)-('QTR BS'!P15-'QTR BS'!O15)-('QTR BS'!P17-'QTR BS'!O17)+('QTR BS'!P22-'QTR BS'!O22)+('QTR BS'!P25-'QTR BS'!O25)+('QTR BS'!P26-'QTR BS'!O26)+('QTR BS'!P27-'QTR BS'!O27)+('QTR BS'!P28-'QTR BS'!O28)+('QTR BS'!P31-'QTR BS'!O31)+('QTR BS'!P32-'QTR BS'!O32)+('QTR BS'!P35-'QTR BS'!O35)+('QTR BS'!P36-'QTR BS'!O36)-('QTR BS'!P3-'QTR BS'!O3)-('QTR BS'!P13-'QTR BS'!O13)-('QTR BS'!P14-'QTR BS'!O14)+('QTR BS'!P33-'QTR BS'!O33)+('QTR BS'!P34-'QTR BS'!O34)</f>
+        <f>-('QTR BS'!P5-'QTR BS'!O5)-('QTR BS'!P8-'QTR BS'!O8)-('QTR BS'!P10-'QTR BS'!O10)-('QTR BS'!P12-'QTR BS'!O12)-('QTR BS'!P15-'QTR BS'!O15)-('QTR BS'!P17-'QTR BS'!O17)+('QTR BS'!P22-'QTR BS'!O22)+('QTR BS'!P25-'QTR BS'!O25)+('QTR BS'!P26-'QTR BS'!O26)+('QTR BS'!P27-'QTR BS'!O27)+('QTR BS'!P28-'QTR BS'!O28)+('QTR BS'!P31-'QTR BS'!O31)+('QTR BS'!P32-'QTR BS'!O32)+('QTR BS'!P35-'QTR BS'!O35)+('QTR BS'!P36-'QTR BS'!O36)-('QTR BS'!P3-'QTR BS'!O3)-('QTR BS'!P13-'QTR BS'!O13)-('QTR BS'!P14-'QTR BS'!O14)+('QTR BS'!P23-'QTR BS'!O23)+('QTR BS'!P33-'QTR BS'!O33)+('QTR BS'!P34-'QTR BS'!O34)</f>
         <v/>
       </c>
       <c r="T15" s="4">
-        <f>-('QTR BS'!Q5-'QTR BS'!P5)-('QTR BS'!Q8-'QTR BS'!P8)-('QTR BS'!Q10-'QTR BS'!P10)-('QTR BS'!Q12-'QTR BS'!P12)-('QTR BS'!Q15-'QTR BS'!P15)-('QTR BS'!Q17-'QTR BS'!P17)+('QTR BS'!Q22-'QTR BS'!P22)+('QTR BS'!Q25-'QTR BS'!P25)+('QTR BS'!Q26-'QTR BS'!P26)+('QTR BS'!Q27-'QTR BS'!P27)+('QTR BS'!Q28-'QTR BS'!P28)+('QTR BS'!Q31-'QTR BS'!P31)+('QTR BS'!Q32-'QTR BS'!P32)+('QTR BS'!Q35-'QTR BS'!P35)+('QTR BS'!Q36-'QTR BS'!P36)-('QTR BS'!Q3-'QTR BS'!P3)-('QTR BS'!Q13-'QTR BS'!P13)-('QTR BS'!Q14-'QTR BS'!P14)+('QTR BS'!Q33-'QTR BS'!P33)+('QTR BS'!Q34-'QTR BS'!P34)</f>
+        <f>-('QTR BS'!Q5-'QTR BS'!P5)-('QTR BS'!Q8-'QTR BS'!P8)-('QTR BS'!Q10-'QTR BS'!P10)-('QTR BS'!Q12-'QTR BS'!P12)-('QTR BS'!Q15-'QTR BS'!P15)-('QTR BS'!Q17-'QTR BS'!P17)+('QTR BS'!Q22-'QTR BS'!P22)+('QTR BS'!Q25-'QTR BS'!P25)+('QTR BS'!Q26-'QTR BS'!P26)+('QTR BS'!Q27-'QTR BS'!P27)+('QTR BS'!Q28-'QTR BS'!P28)+('QTR BS'!Q31-'QTR BS'!P31)+('QTR BS'!Q32-'QTR BS'!P32)+('QTR BS'!Q35-'QTR BS'!P35)+('QTR BS'!Q36-'QTR BS'!P36)-('QTR BS'!Q3-'QTR BS'!P3)-('QTR BS'!Q13-'QTR BS'!P13)-('QTR BS'!Q14-'QTR BS'!P14)+('QTR BS'!Q23-'QTR BS'!P23)+('QTR BS'!Q33-'QTR BS'!P33)+('QTR BS'!Q34-'QTR BS'!P34)</f>
         <v/>
       </c>
       <c r="U15" s="4">
-        <f>-('QTR BS'!R5-'QTR BS'!Q5)-('QTR BS'!R8-'QTR BS'!Q8)-('QTR BS'!R10-'QTR BS'!Q10)-('QTR BS'!R12-'QTR BS'!Q12)-('QTR BS'!R15-'QTR BS'!Q15)-('QTR BS'!R17-'QTR BS'!Q17)+('QTR BS'!R22-'QTR BS'!Q22)+('QTR BS'!R25-'QTR BS'!Q25)+('QTR BS'!R26-'QTR BS'!Q26)+('QTR BS'!R27-'QTR BS'!Q27)+('QTR BS'!R28-'QTR BS'!Q28)+('QTR BS'!R31-'QTR BS'!Q31)+('QTR BS'!R32-'QTR BS'!Q32)+('QTR BS'!R35-'QTR BS'!Q35)+('QTR BS'!R36-'QTR BS'!Q36)-('QTR BS'!R3-'QTR BS'!Q3)-('QTR BS'!R13-'QTR BS'!Q13)-('QTR BS'!R14-'QTR BS'!Q14)+('QTR BS'!R33-'QTR BS'!Q33)+('QTR BS'!R34-'QTR BS'!Q34)</f>
+        <f>-('QTR BS'!R5-'QTR BS'!Q5)-('QTR BS'!R8-'QTR BS'!Q8)-('QTR BS'!R10-'QTR BS'!Q10)-('QTR BS'!R12-'QTR BS'!Q12)-('QTR BS'!R15-'QTR BS'!Q15)-('QTR BS'!R17-'QTR BS'!Q17)+('QTR BS'!R22-'QTR BS'!Q22)+('QTR BS'!R25-'QTR BS'!Q25)+('QTR BS'!R26-'QTR BS'!Q26)+('QTR BS'!R27-'QTR BS'!Q27)+('QTR BS'!R28-'QTR BS'!Q28)+('QTR BS'!R31-'QTR BS'!Q31)+('QTR BS'!R32-'QTR BS'!Q32)+('QTR BS'!R35-'QTR BS'!Q35)+('QTR BS'!R36-'QTR BS'!Q36)-('QTR BS'!R3-'QTR BS'!Q3)-('QTR BS'!R13-'QTR BS'!Q13)-('QTR BS'!R14-'QTR BS'!Q14)+('QTR BS'!R23-'QTR BS'!Q23)+('QTR BS'!R33-'QTR BS'!Q33)+('QTR BS'!R34-'QTR BS'!Q34)</f>
         <v/>
       </c>
       <c r="V15" s="4">
-        <f>-('QTR BS'!S5-'QTR BS'!R5)-('QTR BS'!S8-'QTR BS'!R8)-('QTR BS'!S10-'QTR BS'!R10)-('QTR BS'!S12-'QTR BS'!R12)-('QTR BS'!S15-'QTR BS'!R15)-('QTR BS'!S17-'QTR BS'!R17)+('QTR BS'!S22-'QTR BS'!R22)+('QTR BS'!S25-'QTR BS'!R25)+('QTR BS'!S26-'QTR BS'!R26)+('QTR BS'!S27-'QTR BS'!R27)+('QTR BS'!S28-'QTR BS'!R28)+('QTR BS'!S31-'QTR BS'!R31)+('QTR BS'!S32-'QTR BS'!R32)+('QTR BS'!S35-'QTR BS'!R35)+('QTR BS'!S36-'QTR BS'!R36)-('QTR BS'!S3-'QTR BS'!R3)-('QTR BS'!S13-'QTR BS'!R13)-('QTR BS'!S14-'QTR BS'!R14)+('QTR BS'!S33-'QTR BS'!R33)+('QTR BS'!S34-'QTR BS'!R34)</f>
+        <f>-('QTR BS'!S5-'QTR BS'!R5)-('QTR BS'!S8-'QTR BS'!R8)-('QTR BS'!S10-'QTR BS'!R10)-('QTR BS'!S12-'QTR BS'!R12)-('QTR BS'!S15-'QTR BS'!R15)-('QTR BS'!S17-'QTR BS'!R17)+('QTR BS'!S22-'QTR BS'!R22)+('QTR BS'!S25-'QTR BS'!R25)+('QTR BS'!S26-'QTR BS'!R26)+('QTR BS'!S27-'QTR BS'!R27)+('QTR BS'!S28-'QTR BS'!R28)+('QTR BS'!S31-'QTR BS'!R31)+('QTR BS'!S32-'QTR BS'!R32)+('QTR BS'!S35-'QTR BS'!R35)+('QTR BS'!S36-'QTR BS'!R36)-('QTR BS'!S3-'QTR BS'!R3)-('QTR BS'!S13-'QTR BS'!R13)-('QTR BS'!S14-'QTR BS'!R14)+('QTR BS'!S23-'QTR BS'!R23)+('QTR BS'!S33-'QTR BS'!R33)+('QTR BS'!S34-'QTR BS'!R34)</f>
         <v/>
       </c>
       <c r="W15" s="4">
-        <f>-('QTR BS'!T5-'QTR BS'!S5)-('QTR BS'!T8-'QTR BS'!S8)-('QTR BS'!T10-'QTR BS'!S10)-('QTR BS'!T12-'QTR BS'!S12)-('QTR BS'!T15-'QTR BS'!S15)-('QTR BS'!T17-'QTR BS'!S17)+('QTR BS'!T22-'QTR BS'!S22)+('QTR BS'!T25-'QTR BS'!S25)+('QTR BS'!T26-'QTR BS'!S26)+('QTR BS'!T27-'QTR BS'!S27)+('QTR BS'!T28-'QTR BS'!S28)+('QTR BS'!T31-'QTR BS'!S31)+('QTR BS'!T32-'QTR BS'!S32)+('QTR BS'!T35-'QTR BS'!S35)+('QTR BS'!T36-'QTR BS'!S36)-('QTR BS'!T3-'QTR BS'!S3)-('QTR BS'!T13-'QTR BS'!S13)-('QTR BS'!T14-'QTR BS'!S14)+('QTR BS'!T33-'QTR BS'!S33)+('QTR BS'!T34-'QTR BS'!S34)</f>
+        <f>-('QTR BS'!T5-'QTR BS'!S5)-('QTR BS'!T8-'QTR BS'!S8)-('QTR BS'!T10-'QTR BS'!S10)-('QTR BS'!T12-'QTR BS'!S12)-('QTR BS'!T15-'QTR BS'!S15)-('QTR BS'!T17-'QTR BS'!S17)+('QTR BS'!T22-'QTR BS'!S22)+('QTR BS'!T25-'QTR BS'!S25)+('QTR BS'!T26-'QTR BS'!S26)+('QTR BS'!T27-'QTR BS'!S27)+('QTR BS'!T28-'QTR BS'!S28)+('QTR BS'!T31-'QTR BS'!S31)+('QTR BS'!T32-'QTR BS'!S32)+('QTR BS'!T35-'QTR BS'!S35)+('QTR BS'!T36-'QTR BS'!S36)-('QTR BS'!T3-'QTR BS'!S3)-('QTR BS'!T13-'QTR BS'!S13)-('QTR BS'!T14-'QTR BS'!S14)+('QTR BS'!T23-'QTR BS'!S23)+('QTR BS'!T33-'QTR BS'!S33)+('QTR BS'!T34-'QTR BS'!S34)</f>
         <v/>
       </c>
       <c r="X15" s="4">
-        <f>-('QTR BS'!U5-'QTR BS'!T5)-('QTR BS'!U8-'QTR BS'!T8)-('QTR BS'!U10-'QTR BS'!T10)-('QTR BS'!U12-'QTR BS'!T12)-('QTR BS'!U15-'QTR BS'!T15)-('QTR BS'!U17-'QTR BS'!T17)+('QTR BS'!U22-'QTR BS'!T22)+('QTR BS'!U25-'QTR BS'!T25)+('QTR BS'!U26-'QTR BS'!T26)+('QTR BS'!U27-'QTR BS'!T27)+('QTR BS'!U28-'QTR BS'!T28)+('QTR BS'!U31-'QTR BS'!T31)+('QTR BS'!U32-'QTR BS'!T32)+('QTR BS'!U35-'QTR BS'!T35)+('QTR BS'!U36-'QTR BS'!T36)-('QTR BS'!U3-'QTR BS'!T3)-('QTR BS'!U13-'QTR BS'!T13)-('QTR BS'!U14-'QTR BS'!T14)+('QTR BS'!U33-'QTR BS'!T33)+('QTR BS'!U34-'QTR BS'!T34)</f>
+        <f>-('QTR BS'!U5-'QTR BS'!T5)-('QTR BS'!U8-'QTR BS'!T8)-('QTR BS'!U10-'QTR BS'!T10)-('QTR BS'!U12-'QTR BS'!T12)-('QTR BS'!U15-'QTR BS'!T15)-('QTR BS'!U17-'QTR BS'!T17)+('QTR BS'!U22-'QTR BS'!T22)+('QTR BS'!U25-'QTR BS'!T25)+('QTR BS'!U26-'QTR BS'!T26)+('QTR BS'!U27-'QTR BS'!T27)+('QTR BS'!U28-'QTR BS'!T28)+('QTR BS'!U31-'QTR BS'!T31)+('QTR BS'!U32-'QTR BS'!T32)+('QTR BS'!U35-'QTR BS'!T35)+('QTR BS'!U36-'QTR BS'!T36)-('QTR BS'!U3-'QTR BS'!T3)-('QTR BS'!U13-'QTR BS'!T13)-('QTR BS'!U14-'QTR BS'!T14)+('QTR BS'!U23-'QTR BS'!T23)+('QTR BS'!U33-'QTR BS'!T33)+('QTR BS'!U34-'QTR BS'!T34)</f>
         <v/>
       </c>
       <c r="Y15" s="4">
-        <f>-('QTR BS'!V5-'QTR BS'!U5)-('QTR BS'!V8-'QTR BS'!U8)-('QTR BS'!V10-'QTR BS'!U10)-('QTR BS'!V12-'QTR BS'!U12)-('QTR BS'!V15-'QTR BS'!U15)-('QTR BS'!V17-'QTR BS'!U17)+('QTR BS'!V22-'QTR BS'!U22)+('QTR BS'!V25-'QTR BS'!U25)+('QTR BS'!V26-'QTR BS'!U26)+('QTR BS'!V27-'QTR BS'!U27)+('QTR BS'!V28-'QTR BS'!U28)+('QTR BS'!V31-'QTR BS'!U31)+('QTR BS'!V32-'QTR BS'!U32)+('QTR BS'!V35-'QTR BS'!U35)+('QTR BS'!V36-'QTR BS'!U36)-('QTR BS'!V3-'QTR BS'!U3)-('QTR BS'!V13-'QTR BS'!U13)-('QTR BS'!V14-'QTR BS'!U14)+('QTR BS'!V33-'QTR BS'!U33)+('QTR BS'!V34-'QTR BS'!U34)</f>
+        <f>-('QTR BS'!V5-'QTR BS'!U5)-('QTR BS'!V8-'QTR BS'!U8)-('QTR BS'!V10-'QTR BS'!U10)-('QTR BS'!V12-'QTR BS'!U12)-('QTR BS'!V15-'QTR BS'!U15)-('QTR BS'!V17-'QTR BS'!U17)+('QTR BS'!V22-'QTR BS'!U22)+('QTR BS'!V25-'QTR BS'!U25)+('QTR BS'!V26-'QTR BS'!U26)+('QTR BS'!V27-'QTR BS'!U27)+('QTR BS'!V28-'QTR BS'!U28)+('QTR BS'!V31-'QTR BS'!U31)+('QTR BS'!V32-'QTR BS'!U32)+('QTR BS'!V35-'QTR BS'!U35)+('QTR BS'!V36-'QTR BS'!U36)-('QTR BS'!V3-'QTR BS'!U3)-('QTR BS'!V13-'QTR BS'!U13)-('QTR BS'!V14-'QTR BS'!U14)+('QTR BS'!V23-'QTR BS'!U23)+('QTR BS'!V33-'QTR BS'!U33)+('QTR BS'!V34-'QTR BS'!U34)</f>
         <v/>
       </c>
       <c r="Z15" s="4">
-        <f>-('QTR BS'!W5-'QTR BS'!V5)-('QTR BS'!W8-'QTR BS'!V8)-('QTR BS'!W10-'QTR BS'!V10)-('QTR BS'!W12-'QTR BS'!V12)-('QTR BS'!W15-'QTR BS'!V15)-('QTR BS'!W17-'QTR BS'!V17)+('QTR BS'!W22-'QTR BS'!V22)+('QTR BS'!W25-'QTR BS'!V25)+('QTR BS'!W26-'QTR BS'!V26)+('QTR BS'!W27-'QTR BS'!V27)+('QTR BS'!W28-'QTR BS'!V28)+('QTR BS'!W31-'QTR BS'!V31)+('QTR BS'!W32-'QTR BS'!V32)+('QTR BS'!W35-'QTR BS'!V35)+('QTR BS'!W36-'QTR BS'!V36)-('QTR BS'!W3-'QTR BS'!V3)-('QTR BS'!W13-'QTR BS'!V13)-('QTR BS'!W14-'QTR BS'!V14)+('QTR BS'!W33-'QTR BS'!V33)+('QTR BS'!W34-'QTR BS'!V34)</f>
+        <f>-('QTR BS'!W5-'QTR BS'!V5)-('QTR BS'!W8-'QTR BS'!V8)-('QTR BS'!W10-'QTR BS'!V10)-('QTR BS'!W12-'QTR BS'!V12)-('QTR BS'!W15-'QTR BS'!V15)-('QTR BS'!W17-'QTR BS'!V17)+('QTR BS'!W22-'QTR BS'!V22)+('QTR BS'!W25-'QTR BS'!V25)+('QTR BS'!W26-'QTR BS'!V26)+('QTR BS'!W27-'QTR BS'!V27)+('QTR BS'!W28-'QTR BS'!V28)+('QTR BS'!W31-'QTR BS'!V31)+('QTR BS'!W32-'QTR BS'!V32)+('QTR BS'!W35-'QTR BS'!V35)+('QTR BS'!W36-'QTR BS'!V36)-('QTR BS'!W3-'QTR BS'!V3)-('QTR BS'!W13-'QTR BS'!V13)-('QTR BS'!W14-'QTR BS'!V14)+('QTR BS'!W23-'QTR BS'!V23)+('QTR BS'!W33-'QTR BS'!V33)+('QTR BS'!W34-'QTR BS'!V34)</f>
         <v/>
       </c>
       <c r="AA15" s="4">
-        <f>-('QTR BS'!X5-'QTR BS'!W5)-('QTR BS'!X8-'QTR BS'!W8)-('QTR BS'!X10-'QTR BS'!W10)-('QTR BS'!X12-'QTR BS'!W12)-('QTR BS'!X15-'QTR BS'!W15)-('QTR BS'!X17-'QTR BS'!W17)+('QTR BS'!X22-'QTR BS'!W22)+('QTR BS'!X25-'QTR BS'!W25)+('QTR BS'!X26-'QTR BS'!W26)+('QTR BS'!X27-'QTR BS'!W27)+('QTR BS'!X28-'QTR BS'!W28)+('QTR BS'!X31-'QTR BS'!W31)+('QTR BS'!X32-'QTR BS'!W32)+('QTR BS'!X35-'QTR BS'!W35)+('QTR BS'!X36-'QTR BS'!W36)-('QTR BS'!X3-'QTR BS'!W3)-('QTR BS'!X13-'QTR BS'!W13)-('QTR BS'!X14-'QTR BS'!W14)+('QTR BS'!X33-'QTR BS'!W33)+('QTR BS'!X34-'QTR BS'!W34)</f>
+        <f>-('QTR BS'!X5-'QTR BS'!W5)-('QTR BS'!X8-'QTR BS'!W8)-('QTR BS'!X10-'QTR BS'!W10)-('QTR BS'!X12-'QTR BS'!W12)-('QTR BS'!X15-'QTR BS'!W15)-('QTR BS'!X17-'QTR BS'!W17)+('QTR BS'!X22-'QTR BS'!W22)+('QTR BS'!X25-'QTR BS'!W25)+('QTR BS'!X26-'QTR BS'!W26)+('QTR BS'!X27-'QTR BS'!W27)+('QTR BS'!X28-'QTR BS'!W28)+('QTR BS'!X31-'QTR BS'!W31)+('QTR BS'!X32-'QTR BS'!W32)+('QTR BS'!X35-'QTR BS'!W35)+('QTR BS'!X36-'QTR BS'!W36)-('QTR BS'!X3-'QTR BS'!W3)-('QTR BS'!X13-'QTR BS'!W13)-('QTR BS'!X14-'QTR BS'!W14)+('QTR BS'!X23-'QTR BS'!W23)+('QTR BS'!X33-'QTR BS'!W33)+('QTR BS'!X34-'QTR BS'!W34)</f>
         <v/>
       </c>
       <c r="AB15" s="4">
-        <f>-('QTR BS'!Y5-'QTR BS'!X5)-('QTR BS'!Y8-'QTR BS'!X8)-('QTR BS'!Y10-'QTR BS'!X10)-('QTR BS'!Y12-'QTR BS'!X12)-('QTR BS'!Y15-'QTR BS'!X15)-('QTR BS'!Y17-'QTR BS'!X17)+('QTR BS'!Y22-'QTR BS'!X22)+('QTR BS'!Y25-'QTR BS'!X25)+('QTR BS'!Y26-'QTR BS'!X26)+('QTR BS'!Y27-'QTR BS'!X27)+('QTR BS'!Y28-'QTR BS'!X28)+('QTR BS'!Y31-'QTR BS'!X31)+('QTR BS'!Y32-'QTR BS'!X32)+('QTR BS'!Y35-'QTR BS'!X35)+('QTR BS'!Y36-'QTR BS'!X36)-('QTR BS'!Y3-'QTR BS'!X3)-('QTR BS'!Y13-'QTR BS'!X13)-('QTR BS'!Y14-'QTR BS'!X14)+('QTR BS'!Y33-'QTR BS'!X33)+('QTR BS'!Y34-'QTR BS'!X34)</f>
+        <f>-('QTR BS'!Y5-'QTR BS'!X5)-('QTR BS'!Y8-'QTR BS'!X8)-('QTR BS'!Y10-'QTR BS'!X10)-('QTR BS'!Y12-'QTR BS'!X12)-('QTR BS'!Y15-'QTR BS'!X15)-('QTR BS'!Y17-'QTR BS'!X17)+('QTR BS'!Y22-'QTR BS'!X22)+('QTR BS'!Y25-'QTR BS'!X25)+('QTR BS'!Y26-'QTR BS'!X26)+('QTR BS'!Y27-'QTR BS'!X27)+('QTR BS'!Y28-'QTR BS'!X28)+('QTR BS'!Y31-'QTR BS'!X31)+('QTR BS'!Y32-'QTR BS'!X32)+('QTR BS'!Y35-'QTR BS'!X35)+('QTR BS'!Y36-'QTR BS'!X36)-('QTR BS'!Y3-'QTR BS'!X3)-('QTR BS'!Y13-'QTR BS'!X13)-('QTR BS'!Y14-'QTR BS'!X14)+('QTR BS'!Y23-'QTR BS'!X23)+('QTR BS'!Y33-'QTR BS'!X33)+('QTR BS'!Y34-'QTR BS'!X34)</f>
         <v/>
       </c>
       <c r="AC15" s="4">
-        <f>-('QTR BS'!Z5-'QTR BS'!Y5)-('QTR BS'!Z8-'QTR BS'!Y8)-('QTR BS'!Z10-'QTR BS'!Y10)-('QTR BS'!Z12-'QTR BS'!Y12)-('QTR BS'!Z15-'QTR BS'!Y15)-('QTR BS'!Z17-'QTR BS'!Y17)+('QTR BS'!Z22-'QTR BS'!Y22)+('QTR BS'!Z25-'QTR BS'!Y25)+('QTR BS'!Z26-'QTR BS'!Y26)+('QTR BS'!Z27-'QTR BS'!Y27)+('QTR BS'!Z28-'QTR BS'!Y28)+('QTR BS'!Z31-'QTR BS'!Y31)+('QTR BS'!Z32-'QTR BS'!Y32)+('QTR BS'!Z35-'QTR BS'!Y35)+('QTR BS'!Z36-'QTR BS'!Y36)-('QTR BS'!Z3-'QTR BS'!Y3)-('QTR BS'!Z13-'QTR BS'!Y13)-('QTR BS'!Z14-'QTR BS'!Y14)+('QTR BS'!Z33-'QTR BS'!Y33)+('QTR BS'!Z34-'QTR BS'!Y34)</f>
+        <f>-('QTR BS'!Z5-'QTR BS'!Y5)-('QTR BS'!Z8-'QTR BS'!Y8)-('QTR BS'!Z10-'QTR BS'!Y10)-('QTR BS'!Z12-'QTR BS'!Y12)-('QTR BS'!Z15-'QTR BS'!Y15)-('QTR BS'!Z17-'QTR BS'!Y17)+('QTR BS'!Z22-'QTR BS'!Y22)+('QTR BS'!Z25-'QTR BS'!Y25)+('QTR BS'!Z26-'QTR BS'!Y26)+('QTR BS'!Z27-'QTR BS'!Y27)+('QTR BS'!Z28-'QTR BS'!Y28)+('QTR BS'!Z31-'QTR BS'!Y31)+('QTR BS'!Z32-'QTR BS'!Y32)+('QTR BS'!Z35-'QTR BS'!Y35)+('QTR BS'!Z36-'QTR BS'!Y36)-('QTR BS'!Z3-'QTR BS'!Y3)-('QTR BS'!Z13-'QTR BS'!Y13)-('QTR BS'!Z14-'QTR BS'!Y14)+('QTR BS'!Z23-'QTR BS'!Y23)+('QTR BS'!Z33-'QTR BS'!Y33)+('QTR BS'!Z34-'QTR BS'!Y34)</f>
         <v/>
       </c>
       <c r="AD15" s="4">
-        <f>-('QTR BS'!AA5-'QTR BS'!Z5)-('QTR BS'!AA8-'QTR BS'!Z8)-('QTR BS'!AA10-'QTR BS'!Z10)-('QTR BS'!AA12-'QTR BS'!Z12)-('QTR BS'!AA15-'QTR BS'!Z15)-('QTR BS'!AA17-'QTR BS'!Z17)+('QTR BS'!AA22-'QTR BS'!Z22)+('QTR BS'!AA25-'QTR BS'!Z25)+('QTR BS'!AA26-'QTR BS'!Z26)+('QTR BS'!AA27-'QTR BS'!Z27)+('QTR BS'!AA28-'QTR BS'!Z28)+('QTR BS'!AA31-'QTR BS'!Z31)+('QTR BS'!AA32-'QTR BS'!Z32)+('QTR BS'!AA35-'QTR BS'!Z35)+('QTR BS'!AA36-'QTR BS'!Z36)-('QTR BS'!AA3-'QTR BS'!Z3)-('QTR BS'!AA13-'QTR BS'!Z13)-('QTR BS'!AA14-'QTR BS'!Z14)+('QTR BS'!AA33-'QTR BS'!Z33)+('QTR BS'!AA34-'QTR BS'!Z34)</f>
+        <f>-('QTR BS'!AA5-'QTR BS'!Z5)-('QTR BS'!AA8-'QTR BS'!Z8)-('QTR BS'!AA10-'QTR BS'!Z10)-('QTR BS'!AA12-'QTR BS'!Z12)-('QTR BS'!AA15-'QTR BS'!Z15)-('QTR BS'!AA17-'QTR BS'!Z17)+('QTR BS'!AA22-'QTR BS'!Z22)+('QTR BS'!AA25-'QTR BS'!Z25)+('QTR BS'!AA26-'QTR BS'!Z26)+('QTR BS'!AA27-'QTR BS'!Z27)+('QTR BS'!AA28-'QTR BS'!Z28)+('QTR BS'!AA31-'QTR BS'!Z31)+('QTR BS'!AA32-'QTR BS'!Z32)+('QTR BS'!AA35-'QTR BS'!Z35)+('QTR BS'!AA36-'QTR BS'!Z36)-('QTR BS'!AA3-'QTR BS'!Z3)-('QTR BS'!AA13-'QTR BS'!Z13)-('QTR BS'!AA14-'QTR BS'!Z14)+('QTR BS'!AA23-'QTR BS'!Z23)+('QTR BS'!AA33-'QTR BS'!Z33)+('QTR BS'!AA34-'QTR BS'!Z34)</f>
         <v/>
       </c>
       <c r="AE15" s="4">
-        <f>-('QTR BS'!AB5-'QTR BS'!AA5)-('QTR BS'!AB8-'QTR BS'!AA8)-('QTR BS'!AB10-'QTR BS'!AA10)-('QTR BS'!AB12-'QTR BS'!AA12)-('QTR BS'!AB15-'QTR BS'!AA15)-('QTR BS'!AB17-'QTR BS'!AA17)+('QTR BS'!AB22-'QTR BS'!AA22)+('QTR BS'!AB25-'QTR BS'!AA25)+('QTR BS'!AB26-'QTR BS'!AA26)+('QTR BS'!AB27-'QTR BS'!AA27)+('QTR BS'!AB28-'QTR BS'!AA28)+('QTR BS'!AB31-'QTR BS'!AA31)+('QTR BS'!AB32-'QTR BS'!AA32)+('QTR BS'!AB35-'QTR BS'!AA35)+('QTR BS'!AB36-'QTR BS'!AA36)-('QTR BS'!AB3-'QTR BS'!AA3)-('QTR BS'!AB13-'QTR BS'!AA13)-('QTR BS'!AB14-'QTR BS'!AA14)+('QTR BS'!AB33-'QTR BS'!AA33)+('QTR BS'!AB34-'QTR BS'!AA34)</f>
+        <f>-('QTR BS'!AB5-'QTR BS'!AA5)-('QTR BS'!AB8-'QTR BS'!AA8)-('QTR BS'!AB10-'QTR BS'!AA10)-('QTR BS'!AB12-'QTR BS'!AA12)-('QTR BS'!AB15-'QTR BS'!AA15)-('QTR BS'!AB17-'QTR BS'!AA17)+('QTR BS'!AB22-'QTR BS'!AA22)+('QTR BS'!AB25-'QTR BS'!AA25)+('QTR BS'!AB26-'QTR BS'!AA26)+('QTR BS'!AB27-'QTR BS'!AA27)+('QTR BS'!AB28-'QTR BS'!AA28)+('QTR BS'!AB31-'QTR BS'!AA31)+('QTR BS'!AB32-'QTR BS'!AA32)+('QTR BS'!AB35-'QTR BS'!AA35)+('QTR BS'!AB36-'QTR BS'!AA36)-('QTR BS'!AB3-'QTR BS'!AA3)-('QTR BS'!AB13-'QTR BS'!AA13)-('QTR BS'!AB14-'QTR BS'!AA14)+('QTR BS'!AB23-'QTR BS'!AA23)+('QTR BS'!AB33-'QTR BS'!AA33)+('QTR BS'!AB34-'QTR BS'!AA34)</f>
         <v/>
       </c>
       <c r="AF15" s="4">
-        <f>-('QTR BS'!AC5-'QTR BS'!AB5)-('QTR BS'!AC8-'QTR BS'!AB8)-('QTR BS'!AC10-'QTR BS'!AB10)-('QTR BS'!AC12-'QTR BS'!AB12)-('QTR BS'!AC15-'QTR BS'!AB15)-('QTR BS'!AC17-'QTR BS'!AB17)+('QTR BS'!AC22-'QTR BS'!AB22)+('QTR BS'!AC25-'QTR BS'!AB25)+('QTR BS'!AC26-'QTR BS'!AB26)+('QTR BS'!AC27-'QTR BS'!AB27)+('QTR BS'!AC28-'QTR BS'!AB28)+('QTR BS'!AC31-'QTR BS'!AB31)+('QTR BS'!AC32-'QTR BS'!AB32)+('QTR BS'!AC35-'QTR BS'!AB35)+('QTR BS'!AC36-'QTR BS'!AB36)-('QTR BS'!AC3-'QTR BS'!AB3)-('QTR BS'!AC13-'QTR BS'!AB13)-('QTR BS'!AC14-'QTR BS'!AB14)+('QTR BS'!AC33-'QTR BS'!AB33)+('QTR BS'!AC34-'QTR BS'!AB34)</f>
+        <f>-('QTR BS'!AC5-'QTR BS'!AB5)-('QTR BS'!AC8-'QTR BS'!AB8)-('QTR BS'!AC10-'QTR BS'!AB10)-('QTR BS'!AC12-'QTR BS'!AB12)-('QTR BS'!AC15-'QTR BS'!AB15)-('QTR BS'!AC17-'QTR BS'!AB17)+('QTR BS'!AC22-'QTR BS'!AB22)+('QTR BS'!AC25-'QTR BS'!AB25)+('QTR BS'!AC26-'QTR BS'!AB26)+('QTR BS'!AC27-'QTR BS'!AB27)+('QTR BS'!AC28-'QTR BS'!AB28)+('QTR BS'!AC31-'QTR BS'!AB31)+('QTR BS'!AC32-'QTR BS'!AB32)+('QTR BS'!AC35-'QTR BS'!AB35)+('QTR BS'!AC36-'QTR BS'!AB36)-('QTR BS'!AC3-'QTR BS'!AB3)-('QTR BS'!AC13-'QTR BS'!AB13)-('QTR BS'!AC14-'QTR BS'!AB14)+('QTR BS'!AC23-'QTR BS'!AB23)+('QTR BS'!AC33-'QTR BS'!AB33)+('QTR BS'!AC34-'QTR BS'!AB34)</f>
         <v/>
       </c>
       <c r="AG15" s="4">
-        <f>-('QTR BS'!AD5-'QTR BS'!AC5)-('QTR BS'!AD8-'QTR BS'!AC8)-('QTR BS'!AD10-'QTR BS'!AC10)-('QTR BS'!AD12-'QTR BS'!AC12)-('QTR BS'!AD15-'QTR BS'!AC15)-('QTR BS'!AD17-'QTR BS'!AC17)+('QTR BS'!AD22-'QTR BS'!AC22)+('QTR BS'!AD25-'QTR BS'!AC25)+('QTR BS'!AD26-'QTR BS'!AC26)+('QTR BS'!AD27-'QTR BS'!AC27)+('QTR BS'!AD28-'QTR BS'!AC28)+('QTR BS'!AD31-'QTR BS'!AC31)+('QTR BS'!AD32-'QTR BS'!AC32)+('QTR BS'!AD35-'QTR BS'!AC35)+('QTR BS'!AD36-'QTR BS'!AC36)-('QTR BS'!AD3-'QTR BS'!AC3)-('QTR BS'!AD13-'QTR BS'!AC13)-('QTR BS'!AD14-'QTR BS'!AC14)+('QTR BS'!AD33-'QTR BS'!AC33)+('QTR BS'!AD34-'QTR BS'!AC34)</f>
+        <f>-('QTR BS'!AD5-'QTR BS'!AC5)-('QTR BS'!AD8-'QTR BS'!AC8)-('QTR BS'!AD10-'QTR BS'!AC10)-('QTR BS'!AD12-'QTR BS'!AC12)-('QTR BS'!AD15-'QTR BS'!AC15)-('QTR BS'!AD17-'QTR BS'!AC17)+('QTR BS'!AD22-'QTR BS'!AC22)+('QTR BS'!AD25-'QTR BS'!AC25)+('QTR BS'!AD26-'QTR BS'!AC26)+('QTR BS'!AD27-'QTR BS'!AC27)+('QTR BS'!AD28-'QTR BS'!AC28)+('QTR BS'!AD31-'QTR BS'!AC31)+('QTR BS'!AD32-'QTR BS'!AC32)+('QTR BS'!AD35-'QTR BS'!AC35)+('QTR BS'!AD36-'QTR BS'!AC36)-('QTR BS'!AD3-'QTR BS'!AC3)-('QTR BS'!AD13-'QTR BS'!AC13)-('QTR BS'!AD14-'QTR BS'!AC14)+('QTR BS'!AD23-'QTR BS'!AC23)+('QTR BS'!AD33-'QTR BS'!AC33)+('QTR BS'!AD34-'QTR BS'!AC34)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
vault backup: 2026-04-28 10:40:39
</commit_message>
<xml_diff>
--- a/Knowledge/Model Schema/CELH/Model Output/CELH_model_balance_test.xlsx
+++ b/Knowledge/Model Schema/CELH/Model Output/CELH_model_balance_test.xlsx
@@ -14857,67 +14857,67 @@
         <v/>
       </c>
       <c r="R15" s="4">
-        <f>-('QTR BS'!O5-'QTR BS'!N5)-('QTR BS'!O8-'QTR BS'!N8)-('QTR BS'!O10-'QTR BS'!N10)-('QTR BS'!O12-'QTR BS'!N12)-('QTR BS'!O15-'QTR BS'!N15)-('QTR BS'!O17-'QTR BS'!N17)+('QTR BS'!O22-'QTR BS'!N22)+('QTR BS'!O25-'QTR BS'!N25)+('QTR BS'!O26-'QTR BS'!N26)+('QTR BS'!O27-'QTR BS'!N27)+('QTR BS'!O28-'QTR BS'!N28)+('QTR BS'!O31-'QTR BS'!N31)+('QTR BS'!O32-'QTR BS'!N32)+('QTR BS'!O35-'QTR BS'!N35)+('QTR BS'!O36-'QTR BS'!N36)-('QTR BS'!O3-'QTR BS'!N3)-('QTR BS'!O13-'QTR BS'!N13)-('QTR BS'!O14-'QTR BS'!N14)+('QTR BS'!O23-'QTR BS'!N23)+('QTR BS'!O33-'QTR BS'!N33)+('QTR BS'!O34-'QTR BS'!N34)</f>
+        <f>-('QTR BS'!O5-'QTR BS'!N5)-('QTR BS'!O8-'QTR BS'!N8)-('QTR BS'!O10-'QTR BS'!N10)-('QTR BS'!O12-'QTR BS'!N12)-('QTR BS'!O15-'QTR BS'!N15)-('QTR BS'!O17-'QTR BS'!N17)+('QTR BS'!O22-'QTR BS'!N22)+('QTR BS'!O25-'QTR BS'!N25)+('QTR BS'!O26-'QTR BS'!N26)+('QTR BS'!O27-'QTR BS'!N27)+('QTR BS'!O28-'QTR BS'!N28)+('QTR BS'!O31-'QTR BS'!N31)+('QTR BS'!O32-'QTR BS'!N32)+('QTR BS'!O35-'QTR BS'!N35)+('QTR BS'!O36-'QTR BS'!N36)-('QTR BS'!O3-'QTR BS'!N3)-('QTR BS'!O13-'QTR BS'!N13)-('QTR BS'!O14-'QTR BS'!N14)+('QTR BS'!O23-'QTR BS'!N23)+('QTR BS'!O33-'QTR BS'!N33)+('QTR BS'!O34-'QTR BS'!N34)+('QTR BS'!O39-'QTR BS'!N39)</f>
         <v/>
       </c>
       <c r="S15" s="4">
-        <f>-('QTR BS'!P5-'QTR BS'!O5)-('QTR BS'!P8-'QTR BS'!O8)-('QTR BS'!P10-'QTR BS'!O10)-('QTR BS'!P12-'QTR BS'!O12)-('QTR BS'!P15-'QTR BS'!O15)-('QTR BS'!P17-'QTR BS'!O17)+('QTR BS'!P22-'QTR BS'!O22)+('QTR BS'!P25-'QTR BS'!O25)+('QTR BS'!P26-'QTR BS'!O26)+('QTR BS'!P27-'QTR BS'!O27)+('QTR BS'!P28-'QTR BS'!O28)+('QTR BS'!P31-'QTR BS'!O31)+('QTR BS'!P32-'QTR BS'!O32)+('QTR BS'!P35-'QTR BS'!O35)+('QTR BS'!P36-'QTR BS'!O36)-('QTR BS'!P3-'QTR BS'!O3)-('QTR BS'!P13-'QTR BS'!O13)-('QTR BS'!P14-'QTR BS'!O14)+('QTR BS'!P23-'QTR BS'!O23)+('QTR BS'!P33-'QTR BS'!O33)+('QTR BS'!P34-'QTR BS'!O34)</f>
+        <f>-('QTR BS'!P5-'QTR BS'!O5)-('QTR BS'!P8-'QTR BS'!O8)-('QTR BS'!P10-'QTR BS'!O10)-('QTR BS'!P12-'QTR BS'!O12)-('QTR BS'!P15-'QTR BS'!O15)-('QTR BS'!P17-'QTR BS'!O17)+('QTR BS'!P22-'QTR BS'!O22)+('QTR BS'!P25-'QTR BS'!O25)+('QTR BS'!P26-'QTR BS'!O26)+('QTR BS'!P27-'QTR BS'!O27)+('QTR BS'!P28-'QTR BS'!O28)+('QTR BS'!P31-'QTR BS'!O31)+('QTR BS'!P32-'QTR BS'!O32)+('QTR BS'!P35-'QTR BS'!O35)+('QTR BS'!P36-'QTR BS'!O36)-('QTR BS'!P3-'QTR BS'!O3)-('QTR BS'!P13-'QTR BS'!O13)-('QTR BS'!P14-'QTR BS'!O14)+('QTR BS'!P23-'QTR BS'!O23)+('QTR BS'!P33-'QTR BS'!O33)+('QTR BS'!P34-'QTR BS'!O34)+('QTR BS'!P39-'QTR BS'!O39)</f>
         <v/>
       </c>
       <c r="T15" s="4">
-        <f>-('QTR BS'!Q5-'QTR BS'!P5)-('QTR BS'!Q8-'QTR BS'!P8)-('QTR BS'!Q10-'QTR BS'!P10)-('QTR BS'!Q12-'QTR BS'!P12)-('QTR BS'!Q15-'QTR BS'!P15)-('QTR BS'!Q17-'QTR BS'!P17)+('QTR BS'!Q22-'QTR BS'!P22)+('QTR BS'!Q25-'QTR BS'!P25)+('QTR BS'!Q26-'QTR BS'!P26)+('QTR BS'!Q27-'QTR BS'!P27)+('QTR BS'!Q28-'QTR BS'!P28)+('QTR BS'!Q31-'QTR BS'!P31)+('QTR BS'!Q32-'QTR BS'!P32)+('QTR BS'!Q35-'QTR BS'!P35)+('QTR BS'!Q36-'QTR BS'!P36)-('QTR BS'!Q3-'QTR BS'!P3)-('QTR BS'!Q13-'QTR BS'!P13)-('QTR BS'!Q14-'QTR BS'!P14)+('QTR BS'!Q23-'QTR BS'!P23)+('QTR BS'!Q33-'QTR BS'!P33)+('QTR BS'!Q34-'QTR BS'!P34)</f>
+        <f>-('QTR BS'!Q5-'QTR BS'!P5)-('QTR BS'!Q8-'QTR BS'!P8)-('QTR BS'!Q10-'QTR BS'!P10)-('QTR BS'!Q12-'QTR BS'!P12)-('QTR BS'!Q15-'QTR BS'!P15)-('QTR BS'!Q17-'QTR BS'!P17)+('QTR BS'!Q22-'QTR BS'!P22)+('QTR BS'!Q25-'QTR BS'!P25)+('QTR BS'!Q26-'QTR BS'!P26)+('QTR BS'!Q27-'QTR BS'!P27)+('QTR BS'!Q28-'QTR BS'!P28)+('QTR BS'!Q31-'QTR BS'!P31)+('QTR BS'!Q32-'QTR BS'!P32)+('QTR BS'!Q35-'QTR BS'!P35)+('QTR BS'!Q36-'QTR BS'!P36)-('QTR BS'!Q3-'QTR BS'!P3)-('QTR BS'!Q13-'QTR BS'!P13)-('QTR BS'!Q14-'QTR BS'!P14)+('QTR BS'!Q23-'QTR BS'!P23)+('QTR BS'!Q33-'QTR BS'!P33)+('QTR BS'!Q34-'QTR BS'!P34)+('QTR BS'!Q39-'QTR BS'!P39)</f>
         <v/>
       </c>
       <c r="U15" s="4">
-        <f>-('QTR BS'!R5-'QTR BS'!Q5)-('QTR BS'!R8-'QTR BS'!Q8)-('QTR BS'!R10-'QTR BS'!Q10)-('QTR BS'!R12-'QTR BS'!Q12)-('QTR BS'!R15-'QTR BS'!Q15)-('QTR BS'!R17-'QTR BS'!Q17)+('QTR BS'!R22-'QTR BS'!Q22)+('QTR BS'!R25-'QTR BS'!Q25)+('QTR BS'!R26-'QTR BS'!Q26)+('QTR BS'!R27-'QTR BS'!Q27)+('QTR BS'!R28-'QTR BS'!Q28)+('QTR BS'!R31-'QTR BS'!Q31)+('QTR BS'!R32-'QTR BS'!Q32)+('QTR BS'!R35-'QTR BS'!Q35)+('QTR BS'!R36-'QTR BS'!Q36)-('QTR BS'!R3-'QTR BS'!Q3)-('QTR BS'!R13-'QTR BS'!Q13)-('QTR BS'!R14-'QTR BS'!Q14)+('QTR BS'!R23-'QTR BS'!Q23)+('QTR BS'!R33-'QTR BS'!Q33)+('QTR BS'!R34-'QTR BS'!Q34)</f>
+        <f>-('QTR BS'!R5-'QTR BS'!Q5)-('QTR BS'!R8-'QTR BS'!Q8)-('QTR BS'!R10-'QTR BS'!Q10)-('QTR BS'!R12-'QTR BS'!Q12)-('QTR BS'!R15-'QTR BS'!Q15)-('QTR BS'!R17-'QTR BS'!Q17)+('QTR BS'!R22-'QTR BS'!Q22)+('QTR BS'!R25-'QTR BS'!Q25)+('QTR BS'!R26-'QTR BS'!Q26)+('QTR BS'!R27-'QTR BS'!Q27)+('QTR BS'!R28-'QTR BS'!Q28)+('QTR BS'!R31-'QTR BS'!Q31)+('QTR BS'!R32-'QTR BS'!Q32)+('QTR BS'!R35-'QTR BS'!Q35)+('QTR BS'!R36-'QTR BS'!Q36)-('QTR BS'!R3-'QTR BS'!Q3)-('QTR BS'!R13-'QTR BS'!Q13)-('QTR BS'!R14-'QTR BS'!Q14)+('QTR BS'!R23-'QTR BS'!Q23)+('QTR BS'!R33-'QTR BS'!Q33)+('QTR BS'!R34-'QTR BS'!Q34)+('QTR BS'!R39-'QTR BS'!Q39)</f>
         <v/>
       </c>
       <c r="V15" s="4">
-        <f>-('QTR BS'!S5-'QTR BS'!R5)-('QTR BS'!S8-'QTR BS'!R8)-('QTR BS'!S10-'QTR BS'!R10)-('QTR BS'!S12-'QTR BS'!R12)-('QTR BS'!S15-'QTR BS'!R15)-('QTR BS'!S17-'QTR BS'!R17)+('QTR BS'!S22-'QTR BS'!R22)+('QTR BS'!S25-'QTR BS'!R25)+('QTR BS'!S26-'QTR BS'!R26)+('QTR BS'!S27-'QTR BS'!R27)+('QTR BS'!S28-'QTR BS'!R28)+('QTR BS'!S31-'QTR BS'!R31)+('QTR BS'!S32-'QTR BS'!R32)+('QTR BS'!S35-'QTR BS'!R35)+('QTR BS'!S36-'QTR BS'!R36)-('QTR BS'!S3-'QTR BS'!R3)-('QTR BS'!S13-'QTR BS'!R13)-('QTR BS'!S14-'QTR BS'!R14)+('QTR BS'!S23-'QTR BS'!R23)+('QTR BS'!S33-'QTR BS'!R33)+('QTR BS'!S34-'QTR BS'!R34)</f>
+        <f>-('QTR BS'!S5-'QTR BS'!R5)-('QTR BS'!S8-'QTR BS'!R8)-('QTR BS'!S10-'QTR BS'!R10)-('QTR BS'!S12-'QTR BS'!R12)-('QTR BS'!S15-'QTR BS'!R15)-('QTR BS'!S17-'QTR BS'!R17)+('QTR BS'!S22-'QTR BS'!R22)+('QTR BS'!S25-'QTR BS'!R25)+('QTR BS'!S26-'QTR BS'!R26)+('QTR BS'!S27-'QTR BS'!R27)+('QTR BS'!S28-'QTR BS'!R28)+('QTR BS'!S31-'QTR BS'!R31)+('QTR BS'!S32-'QTR BS'!R32)+('QTR BS'!S35-'QTR BS'!R35)+('QTR BS'!S36-'QTR BS'!R36)-('QTR BS'!S3-'QTR BS'!R3)-('QTR BS'!S13-'QTR BS'!R13)-('QTR BS'!S14-'QTR BS'!R14)+('QTR BS'!S23-'QTR BS'!R23)+('QTR BS'!S33-'QTR BS'!R33)+('QTR BS'!S34-'QTR BS'!R34)+('QTR BS'!S39-'QTR BS'!R39)</f>
         <v/>
       </c>
       <c r="W15" s="4">
-        <f>-('QTR BS'!T5-'QTR BS'!S5)-('QTR BS'!T8-'QTR BS'!S8)-('QTR BS'!T10-'QTR BS'!S10)-('QTR BS'!T12-'QTR BS'!S12)-('QTR BS'!T15-'QTR BS'!S15)-('QTR BS'!T17-'QTR BS'!S17)+('QTR BS'!T22-'QTR BS'!S22)+('QTR BS'!T25-'QTR BS'!S25)+('QTR BS'!T26-'QTR BS'!S26)+('QTR BS'!T27-'QTR BS'!S27)+('QTR BS'!T28-'QTR BS'!S28)+('QTR BS'!T31-'QTR BS'!S31)+('QTR BS'!T32-'QTR BS'!S32)+('QTR BS'!T35-'QTR BS'!S35)+('QTR BS'!T36-'QTR BS'!S36)-('QTR BS'!T3-'QTR BS'!S3)-('QTR BS'!T13-'QTR BS'!S13)-('QTR BS'!T14-'QTR BS'!S14)+('QTR BS'!T23-'QTR BS'!S23)+('QTR BS'!T33-'QTR BS'!S33)+('QTR BS'!T34-'QTR BS'!S34)</f>
+        <f>-('QTR BS'!T5-'QTR BS'!S5)-('QTR BS'!T8-'QTR BS'!S8)-('QTR BS'!T10-'QTR BS'!S10)-('QTR BS'!T12-'QTR BS'!S12)-('QTR BS'!T15-'QTR BS'!S15)-('QTR BS'!T17-'QTR BS'!S17)+('QTR BS'!T22-'QTR BS'!S22)+('QTR BS'!T25-'QTR BS'!S25)+('QTR BS'!T26-'QTR BS'!S26)+('QTR BS'!T27-'QTR BS'!S27)+('QTR BS'!T28-'QTR BS'!S28)+('QTR BS'!T31-'QTR BS'!S31)+('QTR BS'!T32-'QTR BS'!S32)+('QTR BS'!T35-'QTR BS'!S35)+('QTR BS'!T36-'QTR BS'!S36)-('QTR BS'!T3-'QTR BS'!S3)-('QTR BS'!T13-'QTR BS'!S13)-('QTR BS'!T14-'QTR BS'!S14)+('QTR BS'!T23-'QTR BS'!S23)+('QTR BS'!T33-'QTR BS'!S33)+('QTR BS'!T34-'QTR BS'!S34)+('QTR BS'!T39-'QTR BS'!S39)</f>
         <v/>
       </c>
       <c r="X15" s="4">
-        <f>-('QTR BS'!U5-'QTR BS'!T5)-('QTR BS'!U8-'QTR BS'!T8)-('QTR BS'!U10-'QTR BS'!T10)-('QTR BS'!U12-'QTR BS'!T12)-('QTR BS'!U15-'QTR BS'!T15)-('QTR BS'!U17-'QTR BS'!T17)+('QTR BS'!U22-'QTR BS'!T22)+('QTR BS'!U25-'QTR BS'!T25)+('QTR BS'!U26-'QTR BS'!T26)+('QTR BS'!U27-'QTR BS'!T27)+('QTR BS'!U28-'QTR BS'!T28)+('QTR BS'!U31-'QTR BS'!T31)+('QTR BS'!U32-'QTR BS'!T32)+('QTR BS'!U35-'QTR BS'!T35)+('QTR BS'!U36-'QTR BS'!T36)-('QTR BS'!U3-'QTR BS'!T3)-('QTR BS'!U13-'QTR BS'!T13)-('QTR BS'!U14-'QTR BS'!T14)+('QTR BS'!U23-'QTR BS'!T23)+('QTR BS'!U33-'QTR BS'!T33)+('QTR BS'!U34-'QTR BS'!T34)</f>
+        <f>-('QTR BS'!U5-'QTR BS'!T5)-('QTR BS'!U8-'QTR BS'!T8)-('QTR BS'!U10-'QTR BS'!T10)-('QTR BS'!U12-'QTR BS'!T12)-('QTR BS'!U15-'QTR BS'!T15)-('QTR BS'!U17-'QTR BS'!T17)+('QTR BS'!U22-'QTR BS'!T22)+('QTR BS'!U25-'QTR BS'!T25)+('QTR BS'!U26-'QTR BS'!T26)+('QTR BS'!U27-'QTR BS'!T27)+('QTR BS'!U28-'QTR BS'!T28)+('QTR BS'!U31-'QTR BS'!T31)+('QTR BS'!U32-'QTR BS'!T32)+('QTR BS'!U35-'QTR BS'!T35)+('QTR BS'!U36-'QTR BS'!T36)-('QTR BS'!U3-'QTR BS'!T3)-('QTR BS'!U13-'QTR BS'!T13)-('QTR BS'!U14-'QTR BS'!T14)+('QTR BS'!U23-'QTR BS'!T23)+('QTR BS'!U33-'QTR BS'!T33)+('QTR BS'!U34-'QTR BS'!T34)+('QTR BS'!U39-'QTR BS'!T39)</f>
         <v/>
       </c>
       <c r="Y15" s="4">
-        <f>-('QTR BS'!V5-'QTR BS'!U5)-('QTR BS'!V8-'QTR BS'!U8)-('QTR BS'!V10-'QTR BS'!U10)-('QTR BS'!V12-'QTR BS'!U12)-('QTR BS'!V15-'QTR BS'!U15)-('QTR BS'!V17-'QTR BS'!U17)+('QTR BS'!V22-'QTR BS'!U22)+('QTR BS'!V25-'QTR BS'!U25)+('QTR BS'!V26-'QTR BS'!U26)+('QTR BS'!V27-'QTR BS'!U27)+('QTR BS'!V28-'QTR BS'!U28)+('QTR BS'!V31-'QTR BS'!U31)+('QTR BS'!V32-'QTR BS'!U32)+('QTR BS'!V35-'QTR BS'!U35)+('QTR BS'!V36-'QTR BS'!U36)-('QTR BS'!V3-'QTR BS'!U3)-('QTR BS'!V13-'QTR BS'!U13)-('QTR BS'!V14-'QTR BS'!U14)+('QTR BS'!V23-'QTR BS'!U23)+('QTR BS'!V33-'QTR BS'!U33)+('QTR BS'!V34-'QTR BS'!U34)</f>
+        <f>-('QTR BS'!V5-'QTR BS'!U5)-('QTR BS'!V8-'QTR BS'!U8)-('QTR BS'!V10-'QTR BS'!U10)-('QTR BS'!V12-'QTR BS'!U12)-('QTR BS'!V15-'QTR BS'!U15)-('QTR BS'!V17-'QTR BS'!U17)+('QTR BS'!V22-'QTR BS'!U22)+('QTR BS'!V25-'QTR BS'!U25)+('QTR BS'!V26-'QTR BS'!U26)+('QTR BS'!V27-'QTR BS'!U27)+('QTR BS'!V28-'QTR BS'!U28)+('QTR BS'!V31-'QTR BS'!U31)+('QTR BS'!V32-'QTR BS'!U32)+('QTR BS'!V35-'QTR BS'!U35)+('QTR BS'!V36-'QTR BS'!U36)-('QTR BS'!V3-'QTR BS'!U3)-('QTR BS'!V13-'QTR BS'!U13)-('QTR BS'!V14-'QTR BS'!U14)+('QTR BS'!V23-'QTR BS'!U23)+('QTR BS'!V33-'QTR BS'!U33)+('QTR BS'!V34-'QTR BS'!U34)+('QTR BS'!V39-'QTR BS'!U39)</f>
         <v/>
       </c>
       <c r="Z15" s="4">
-        <f>-('QTR BS'!W5-'QTR BS'!V5)-('QTR BS'!W8-'QTR BS'!V8)-('QTR BS'!W10-'QTR BS'!V10)-('QTR BS'!W12-'QTR BS'!V12)-('QTR BS'!W15-'QTR BS'!V15)-('QTR BS'!W17-'QTR BS'!V17)+('QTR BS'!W22-'QTR BS'!V22)+('QTR BS'!W25-'QTR BS'!V25)+('QTR BS'!W26-'QTR BS'!V26)+('QTR BS'!W27-'QTR BS'!V27)+('QTR BS'!W28-'QTR BS'!V28)+('QTR BS'!W31-'QTR BS'!V31)+('QTR BS'!W32-'QTR BS'!V32)+('QTR BS'!W35-'QTR BS'!V35)+('QTR BS'!W36-'QTR BS'!V36)-('QTR BS'!W3-'QTR BS'!V3)-('QTR BS'!W13-'QTR BS'!V13)-('QTR BS'!W14-'QTR BS'!V14)+('QTR BS'!W23-'QTR BS'!V23)+('QTR BS'!W33-'QTR BS'!V33)+('QTR BS'!W34-'QTR BS'!V34)</f>
+        <f>-('QTR BS'!W5-'QTR BS'!V5)-('QTR BS'!W8-'QTR BS'!V8)-('QTR BS'!W10-'QTR BS'!V10)-('QTR BS'!W12-'QTR BS'!V12)-('QTR BS'!W15-'QTR BS'!V15)-('QTR BS'!W17-'QTR BS'!V17)+('QTR BS'!W22-'QTR BS'!V22)+('QTR BS'!W25-'QTR BS'!V25)+('QTR BS'!W26-'QTR BS'!V26)+('QTR BS'!W27-'QTR BS'!V27)+('QTR BS'!W28-'QTR BS'!V28)+('QTR BS'!W31-'QTR BS'!V31)+('QTR BS'!W32-'QTR BS'!V32)+('QTR BS'!W35-'QTR BS'!V35)+('QTR BS'!W36-'QTR BS'!V36)-('QTR BS'!W3-'QTR BS'!V3)-('QTR BS'!W13-'QTR BS'!V13)-('QTR BS'!W14-'QTR BS'!V14)+('QTR BS'!W23-'QTR BS'!V23)+('QTR BS'!W33-'QTR BS'!V33)+('QTR BS'!W34-'QTR BS'!V34)+('QTR BS'!W39-'QTR BS'!V39)</f>
         <v/>
       </c>
       <c r="AA15" s="4">
-        <f>-('QTR BS'!X5-'QTR BS'!W5)-('QTR BS'!X8-'QTR BS'!W8)-('QTR BS'!X10-'QTR BS'!W10)-('QTR BS'!X12-'QTR BS'!W12)-('QTR BS'!X15-'QTR BS'!W15)-('QTR BS'!X17-'QTR BS'!W17)+('QTR BS'!X22-'QTR BS'!W22)+('QTR BS'!X25-'QTR BS'!W25)+('QTR BS'!X26-'QTR BS'!W26)+('QTR BS'!X27-'QTR BS'!W27)+('QTR BS'!X28-'QTR BS'!W28)+('QTR BS'!X31-'QTR BS'!W31)+('QTR BS'!X32-'QTR BS'!W32)+('QTR BS'!X35-'QTR BS'!W35)+('QTR BS'!X36-'QTR BS'!W36)-('QTR BS'!X3-'QTR BS'!W3)-('QTR BS'!X13-'QTR BS'!W13)-('QTR BS'!X14-'QTR BS'!W14)+('QTR BS'!X23-'QTR BS'!W23)+('QTR BS'!X33-'QTR BS'!W33)+('QTR BS'!X34-'QTR BS'!W34)</f>
+        <f>-('QTR BS'!X5-'QTR BS'!W5)-('QTR BS'!X8-'QTR BS'!W8)-('QTR BS'!X10-'QTR BS'!W10)-('QTR BS'!X12-'QTR BS'!W12)-('QTR BS'!X15-'QTR BS'!W15)-('QTR BS'!X17-'QTR BS'!W17)+('QTR BS'!X22-'QTR BS'!W22)+('QTR BS'!X25-'QTR BS'!W25)+('QTR BS'!X26-'QTR BS'!W26)+('QTR BS'!X27-'QTR BS'!W27)+('QTR BS'!X28-'QTR BS'!W28)+('QTR BS'!X31-'QTR BS'!W31)+('QTR BS'!X32-'QTR BS'!W32)+('QTR BS'!X35-'QTR BS'!W35)+('QTR BS'!X36-'QTR BS'!W36)-('QTR BS'!X3-'QTR BS'!W3)-('QTR BS'!X13-'QTR BS'!W13)-('QTR BS'!X14-'QTR BS'!W14)+('QTR BS'!X23-'QTR BS'!W23)+('QTR BS'!X33-'QTR BS'!W33)+('QTR BS'!X34-'QTR BS'!W34)+('QTR BS'!X39-'QTR BS'!W39)</f>
         <v/>
       </c>
       <c r="AB15" s="4">
-        <f>-('QTR BS'!Y5-'QTR BS'!X5)-('QTR BS'!Y8-'QTR BS'!X8)-('QTR BS'!Y10-'QTR BS'!X10)-('QTR BS'!Y12-'QTR BS'!X12)-('QTR BS'!Y15-'QTR BS'!X15)-('QTR BS'!Y17-'QTR BS'!X17)+('QTR BS'!Y22-'QTR BS'!X22)+('QTR BS'!Y25-'QTR BS'!X25)+('QTR BS'!Y26-'QTR BS'!X26)+('QTR BS'!Y27-'QTR BS'!X27)+('QTR BS'!Y28-'QTR BS'!X28)+('QTR BS'!Y31-'QTR BS'!X31)+('QTR BS'!Y32-'QTR BS'!X32)+('QTR BS'!Y35-'QTR BS'!X35)+('QTR BS'!Y36-'QTR BS'!X36)-('QTR BS'!Y3-'QTR BS'!X3)-('QTR BS'!Y13-'QTR BS'!X13)-('QTR BS'!Y14-'QTR BS'!X14)+('QTR BS'!Y23-'QTR BS'!X23)+('QTR BS'!Y33-'QTR BS'!X33)+('QTR BS'!Y34-'QTR BS'!X34)</f>
+        <f>-('QTR BS'!Y5-'QTR BS'!X5)-('QTR BS'!Y8-'QTR BS'!X8)-('QTR BS'!Y10-'QTR BS'!X10)-('QTR BS'!Y12-'QTR BS'!X12)-('QTR BS'!Y15-'QTR BS'!X15)-('QTR BS'!Y17-'QTR BS'!X17)+('QTR BS'!Y22-'QTR BS'!X22)+('QTR BS'!Y25-'QTR BS'!X25)+('QTR BS'!Y26-'QTR BS'!X26)+('QTR BS'!Y27-'QTR BS'!X27)+('QTR BS'!Y28-'QTR BS'!X28)+('QTR BS'!Y31-'QTR BS'!X31)+('QTR BS'!Y32-'QTR BS'!X32)+('QTR BS'!Y35-'QTR BS'!X35)+('QTR BS'!Y36-'QTR BS'!X36)-('QTR BS'!Y3-'QTR BS'!X3)-('QTR BS'!Y13-'QTR BS'!X13)-('QTR BS'!Y14-'QTR BS'!X14)+('QTR BS'!Y23-'QTR BS'!X23)+('QTR BS'!Y33-'QTR BS'!X33)+('QTR BS'!Y34-'QTR BS'!X34)+('QTR BS'!Y39-'QTR BS'!X39)</f>
         <v/>
       </c>
       <c r="AC15" s="4">
-        <f>-('QTR BS'!Z5-'QTR BS'!Y5)-('QTR BS'!Z8-'QTR BS'!Y8)-('QTR BS'!Z10-'QTR BS'!Y10)-('QTR BS'!Z12-'QTR BS'!Y12)-('QTR BS'!Z15-'QTR BS'!Y15)-('QTR BS'!Z17-'QTR BS'!Y17)+('QTR BS'!Z22-'QTR BS'!Y22)+('QTR BS'!Z25-'QTR BS'!Y25)+('QTR BS'!Z26-'QTR BS'!Y26)+('QTR BS'!Z27-'QTR BS'!Y27)+('QTR BS'!Z28-'QTR BS'!Y28)+('QTR BS'!Z31-'QTR BS'!Y31)+('QTR BS'!Z32-'QTR BS'!Y32)+('QTR BS'!Z35-'QTR BS'!Y35)+('QTR BS'!Z36-'QTR BS'!Y36)-('QTR BS'!Z3-'QTR BS'!Y3)-('QTR BS'!Z13-'QTR BS'!Y13)-('QTR BS'!Z14-'QTR BS'!Y14)+('QTR BS'!Z23-'QTR BS'!Y23)+('QTR BS'!Z33-'QTR BS'!Y33)+('QTR BS'!Z34-'QTR BS'!Y34)</f>
+        <f>-('QTR BS'!Z5-'QTR BS'!Y5)-('QTR BS'!Z8-'QTR BS'!Y8)-('QTR BS'!Z10-'QTR BS'!Y10)-('QTR BS'!Z12-'QTR BS'!Y12)-('QTR BS'!Z15-'QTR BS'!Y15)-('QTR BS'!Z17-'QTR BS'!Y17)+('QTR BS'!Z22-'QTR BS'!Y22)+('QTR BS'!Z25-'QTR BS'!Y25)+('QTR BS'!Z26-'QTR BS'!Y26)+('QTR BS'!Z27-'QTR BS'!Y27)+('QTR BS'!Z28-'QTR BS'!Y28)+('QTR BS'!Z31-'QTR BS'!Y31)+('QTR BS'!Z32-'QTR BS'!Y32)+('QTR BS'!Z35-'QTR BS'!Y35)+('QTR BS'!Z36-'QTR BS'!Y36)-('QTR BS'!Z3-'QTR BS'!Y3)-('QTR BS'!Z13-'QTR BS'!Y13)-('QTR BS'!Z14-'QTR BS'!Y14)+('QTR BS'!Z23-'QTR BS'!Y23)+('QTR BS'!Z33-'QTR BS'!Y33)+('QTR BS'!Z34-'QTR BS'!Y34)+('QTR BS'!Z39-'QTR BS'!Y39)</f>
         <v/>
       </c>
       <c r="AD15" s="4">
-        <f>-('QTR BS'!AA5-'QTR BS'!Z5)-('QTR BS'!AA8-'QTR BS'!Z8)-('QTR BS'!AA10-'QTR BS'!Z10)-('QTR BS'!AA12-'QTR BS'!Z12)-('QTR BS'!AA15-'QTR BS'!Z15)-('QTR BS'!AA17-'QTR BS'!Z17)+('QTR BS'!AA22-'QTR BS'!Z22)+('QTR BS'!AA25-'QTR BS'!Z25)+('QTR BS'!AA26-'QTR BS'!Z26)+('QTR BS'!AA27-'QTR BS'!Z27)+('QTR BS'!AA28-'QTR BS'!Z28)+('QTR BS'!AA31-'QTR BS'!Z31)+('QTR BS'!AA32-'QTR BS'!Z32)+('QTR BS'!AA35-'QTR BS'!Z35)+('QTR BS'!AA36-'QTR BS'!Z36)-('QTR BS'!AA3-'QTR BS'!Z3)-('QTR BS'!AA13-'QTR BS'!Z13)-('QTR BS'!AA14-'QTR BS'!Z14)+('QTR BS'!AA23-'QTR BS'!Z23)+('QTR BS'!AA33-'QTR BS'!Z33)+('QTR BS'!AA34-'QTR BS'!Z34)</f>
+        <f>-('QTR BS'!AA5-'QTR BS'!Z5)-('QTR BS'!AA8-'QTR BS'!Z8)-('QTR BS'!AA10-'QTR BS'!Z10)-('QTR BS'!AA12-'QTR BS'!Z12)-('QTR BS'!AA15-'QTR BS'!Z15)-('QTR BS'!AA17-'QTR BS'!Z17)+('QTR BS'!AA22-'QTR BS'!Z22)+('QTR BS'!AA25-'QTR BS'!Z25)+('QTR BS'!AA26-'QTR BS'!Z26)+('QTR BS'!AA27-'QTR BS'!Z27)+('QTR BS'!AA28-'QTR BS'!Z28)+('QTR BS'!AA31-'QTR BS'!Z31)+('QTR BS'!AA32-'QTR BS'!Z32)+('QTR BS'!AA35-'QTR BS'!Z35)+('QTR BS'!AA36-'QTR BS'!Z36)-('QTR BS'!AA3-'QTR BS'!Z3)-('QTR BS'!AA13-'QTR BS'!Z13)-('QTR BS'!AA14-'QTR BS'!Z14)+('QTR BS'!AA23-'QTR BS'!Z23)+('QTR BS'!AA33-'QTR BS'!Z33)+('QTR BS'!AA34-'QTR BS'!Z34)+('QTR BS'!AA39-'QTR BS'!Z39)</f>
         <v/>
       </c>
       <c r="AE15" s="4">
-        <f>-('QTR BS'!AB5-'QTR BS'!AA5)-('QTR BS'!AB8-'QTR BS'!AA8)-('QTR BS'!AB10-'QTR BS'!AA10)-('QTR BS'!AB12-'QTR BS'!AA12)-('QTR BS'!AB15-'QTR BS'!AA15)-('QTR BS'!AB17-'QTR BS'!AA17)+('QTR BS'!AB22-'QTR BS'!AA22)+('QTR BS'!AB25-'QTR BS'!AA25)+('QTR BS'!AB26-'QTR BS'!AA26)+('QTR BS'!AB27-'QTR BS'!AA27)+('QTR BS'!AB28-'QTR BS'!AA28)+('QTR BS'!AB31-'QTR BS'!AA31)+('QTR BS'!AB32-'QTR BS'!AA32)+('QTR BS'!AB35-'QTR BS'!AA35)+('QTR BS'!AB36-'QTR BS'!AA36)-('QTR BS'!AB3-'QTR BS'!AA3)-('QTR BS'!AB13-'QTR BS'!AA13)-('QTR BS'!AB14-'QTR BS'!AA14)+('QTR BS'!AB23-'QTR BS'!AA23)+('QTR BS'!AB33-'QTR BS'!AA33)+('QTR BS'!AB34-'QTR BS'!AA34)</f>
+        <f>-('QTR BS'!AB5-'QTR BS'!AA5)-('QTR BS'!AB8-'QTR BS'!AA8)-('QTR BS'!AB10-'QTR BS'!AA10)-('QTR BS'!AB12-'QTR BS'!AA12)-('QTR BS'!AB15-'QTR BS'!AA15)-('QTR BS'!AB17-'QTR BS'!AA17)+('QTR BS'!AB22-'QTR BS'!AA22)+('QTR BS'!AB25-'QTR BS'!AA25)+('QTR BS'!AB26-'QTR BS'!AA26)+('QTR BS'!AB27-'QTR BS'!AA27)+('QTR BS'!AB28-'QTR BS'!AA28)+('QTR BS'!AB31-'QTR BS'!AA31)+('QTR BS'!AB32-'QTR BS'!AA32)+('QTR BS'!AB35-'QTR BS'!AA35)+('QTR BS'!AB36-'QTR BS'!AA36)-('QTR BS'!AB3-'QTR BS'!AA3)-('QTR BS'!AB13-'QTR BS'!AA13)-('QTR BS'!AB14-'QTR BS'!AA14)+('QTR BS'!AB23-'QTR BS'!AA23)+('QTR BS'!AB33-'QTR BS'!AA33)+('QTR BS'!AB34-'QTR BS'!AA34)+('QTR BS'!AB39-'QTR BS'!AA39)</f>
         <v/>
       </c>
       <c r="AF15" s="4">
-        <f>-('QTR BS'!AC5-'QTR BS'!AB5)-('QTR BS'!AC8-'QTR BS'!AB8)-('QTR BS'!AC10-'QTR BS'!AB10)-('QTR BS'!AC12-'QTR BS'!AB12)-('QTR BS'!AC15-'QTR BS'!AB15)-('QTR BS'!AC17-'QTR BS'!AB17)+('QTR BS'!AC22-'QTR BS'!AB22)+('QTR BS'!AC25-'QTR BS'!AB25)+('QTR BS'!AC26-'QTR BS'!AB26)+('QTR BS'!AC27-'QTR BS'!AB27)+('QTR BS'!AC28-'QTR BS'!AB28)+('QTR BS'!AC31-'QTR BS'!AB31)+('QTR BS'!AC32-'QTR BS'!AB32)+('QTR BS'!AC35-'QTR BS'!AB35)+('QTR BS'!AC36-'QTR BS'!AB36)-('QTR BS'!AC3-'QTR BS'!AB3)-('QTR BS'!AC13-'QTR BS'!AB13)-('QTR BS'!AC14-'QTR BS'!AB14)+('QTR BS'!AC23-'QTR BS'!AB23)+('QTR BS'!AC33-'QTR BS'!AB33)+('QTR BS'!AC34-'QTR BS'!AB34)</f>
+        <f>-('QTR BS'!AC5-'QTR BS'!AB5)-('QTR BS'!AC8-'QTR BS'!AB8)-('QTR BS'!AC10-'QTR BS'!AB10)-('QTR BS'!AC12-'QTR BS'!AB12)-('QTR BS'!AC15-'QTR BS'!AB15)-('QTR BS'!AC17-'QTR BS'!AB17)+('QTR BS'!AC22-'QTR BS'!AB22)+('QTR BS'!AC25-'QTR BS'!AB25)+('QTR BS'!AC26-'QTR BS'!AB26)+('QTR BS'!AC27-'QTR BS'!AB27)+('QTR BS'!AC28-'QTR BS'!AB28)+('QTR BS'!AC31-'QTR BS'!AB31)+('QTR BS'!AC32-'QTR BS'!AB32)+('QTR BS'!AC35-'QTR BS'!AB35)+('QTR BS'!AC36-'QTR BS'!AB36)-('QTR BS'!AC3-'QTR BS'!AB3)-('QTR BS'!AC13-'QTR BS'!AB13)-('QTR BS'!AC14-'QTR BS'!AB14)+('QTR BS'!AC23-'QTR BS'!AB23)+('QTR BS'!AC33-'QTR BS'!AB33)+('QTR BS'!AC34-'QTR BS'!AB34)+('QTR BS'!AC39-'QTR BS'!AB39)</f>
         <v/>
       </c>
       <c r="AG15" s="4">
-        <f>-('QTR BS'!AD5-'QTR BS'!AC5)-('QTR BS'!AD8-'QTR BS'!AC8)-('QTR BS'!AD10-'QTR BS'!AC10)-('QTR BS'!AD12-'QTR BS'!AC12)-('QTR BS'!AD15-'QTR BS'!AC15)-('QTR BS'!AD17-'QTR BS'!AC17)+('QTR BS'!AD22-'QTR BS'!AC22)+('QTR BS'!AD25-'QTR BS'!AC25)+('QTR BS'!AD26-'QTR BS'!AC26)+('QTR BS'!AD27-'QTR BS'!AC27)+('QTR BS'!AD28-'QTR BS'!AC28)+('QTR BS'!AD31-'QTR BS'!AC31)+('QTR BS'!AD32-'QTR BS'!AC32)+('QTR BS'!AD35-'QTR BS'!AC35)+('QTR BS'!AD36-'QTR BS'!AC36)-('QTR BS'!AD3-'QTR BS'!AC3)-('QTR BS'!AD13-'QTR BS'!AC13)-('QTR BS'!AD14-'QTR BS'!AC14)+('QTR BS'!AD23-'QTR BS'!AC23)+('QTR BS'!AD33-'QTR BS'!AC33)+('QTR BS'!AD34-'QTR BS'!AC34)</f>
+        <f>-('QTR BS'!AD5-'QTR BS'!AC5)-('QTR BS'!AD8-'QTR BS'!AC8)-('QTR BS'!AD10-'QTR BS'!AC10)-('QTR BS'!AD12-'QTR BS'!AC12)-('QTR BS'!AD15-'QTR BS'!AC15)-('QTR BS'!AD17-'QTR BS'!AC17)+('QTR BS'!AD22-'QTR BS'!AC22)+('QTR BS'!AD25-'QTR BS'!AC25)+('QTR BS'!AD26-'QTR BS'!AC26)+('QTR BS'!AD27-'QTR BS'!AC27)+('QTR BS'!AD28-'QTR BS'!AC28)+('QTR BS'!AD31-'QTR BS'!AC31)+('QTR BS'!AD32-'QTR BS'!AC32)+('QTR BS'!AD35-'QTR BS'!AC35)+('QTR BS'!AD36-'QTR BS'!AC36)-('QTR BS'!AD3-'QTR BS'!AC3)-('QTR BS'!AD13-'QTR BS'!AC13)-('QTR BS'!AD14-'QTR BS'!AC14)+('QTR BS'!AD23-'QTR BS'!AC23)+('QTR BS'!AD33-'QTR BS'!AC33)+('QTR BS'!AD34-'QTR BS'!AC34)+('QTR BS'!AD39-'QTR BS'!AC39)</f>
         <v/>
       </c>
     </row>

</xml_diff>